<commit_message>
versão ETC + DOE-TCESP
</commit_message>
<xml_diff>
--- a/sp_aguas.xlsx
+++ b/sp_aguas.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="usuarios" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="demandas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="historico" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="usuarios" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demandas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="historico" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'usuarios'!$A$1:$I$2</definedName>
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -628,6 +628,41 @@
           <t>atualizado_em</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>numero_etc</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>doe_data</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>doe_edicao</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>doe_secao</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>doe_palavra_chave</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>doe_publicacao</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>doe_url</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -653,8 +688,6 @@
           <t>CD4</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>2026-09-10</t>
@@ -675,7 +708,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>1</v>
       </c>
@@ -815,9 +847,6 @@
           <t>ETC - Contrato 2025 / TC - 016645.989.26-0 (Termo Aditivo)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>2026-09-15</t>
@@ -838,7 +867,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>1</v>
       </c>

</xml_diff>